<commit_message>
Deploying to gh-pages from @ mattaq31/Hash-CAD@9006c3a0d6484c3ddd48229ce97ddaad89c2a58d 🚀
</commit_message>
<xml_diff>
--- a/plates/cargo_plates/sw_src010_nelson_quimby_bart_edna_maxed.xlsx
+++ b/plates/cargo_plates/sw_src010_nelson_quimby_bart_edna_maxed.xlsx
@@ -1,22 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/matt/Documents/Shih_Lab_Postdoc/research_projects/crisscross_code/crisscross_kit/crisscross/dna_source_plates/cargo_plates/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27E4C657-E5B5-F345-BE7F-D15A67240173}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="50440" windowHeight="28180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="All Data" sheetId="1" r:id="rId1"/>
     <sheet name="2D Layout" sheetId="2" r:id="rId2"/>
     <sheet name="2D Label" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2007" uniqueCount="1007">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1751" uniqueCount="1103">
   <si>
     <t>well</t>
   </si>
@@ -3037,13 +3043,301 @@
   </si>
   <si>
     <t>X</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h5-position_1</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h5-position_2</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h5-position_3</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h5-position_4</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h5-position_5</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h5-position_6</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h5-position_7</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h5-position_8</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h5-position_9</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h5-position_10</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h5-position_11</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h5-position_12</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h5-position_13</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h5-position_14</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h5-position_15</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h5-position_16</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h5-position_17</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h5-position_18</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h5-position_19</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h5-position_20</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h5-position_21</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h5-position_22</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h5-position_23</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h5-position_24</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h5-position_25</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h5-position_26</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h5-position_27</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h5-position_28</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h5-position_29</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h5-position_30</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h5-position_31</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h5-position_32</t>
+  </si>
+  <si>
+    <t>CCTGGCCCTCTCCAACGTCAAAGGGCGACTTGACGGGGAAAGttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>CATAAAGTGGTGAGACGGGCAACAGCTGAGAAAGCGAAAGGAttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>TCTGTGGTGGCTCACAATTCCACACAACCGGTCACGCTGCGCttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>ATCCGCCGGGATCCAGCGCAGTGTCACTCGCCGCTACAGGGCttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>TTTTCGTCTTCAGCGGGGTCATTGCAGGTATAACGTGCTTTCttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>TTTCTCCGTTGCTGATTGCCGTTCCGGCAGGAGGCCGATTAAttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>GCTATTACGGTTTACCAGTCCCGGAATTGAATCCTGAGAAGTttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>GACCGTAATCTGTTGGGAAGGGCGATCGAAAAGAGTCTGTCCttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>GGAAGATTGCGTCGGATTCTCCGTGGGACTTCTTTGATTAGTttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>AGACAGTCACCCCGGTTGATAATCAGAACTCAAACTATCGGCttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>GGCAAGGCATAGGTAAAGATTCAAAAGGCCGCCAGCCATTGCttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>AATATGCAATAGTAGTAGCATTAACATCACATTTTGACGCTCttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>AGCGGATTGGCTGAATATAATGCTGTAGGCAGATTCACCAGTttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>GATAAAAACGGTCTTTACCCTGACTATTTGGCCAACAGAGATttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>TAAGAACTGCAACACTATCATAACCCTCATACGTGGCACAGAttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>ACGGTGTACACTTTAATCATTGTGAATTAATGCGCGAACTGAttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>ACGAAAGAGCCGAACTGACCAACTTTGACCGAACGAACCACCttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>CGCCCACGCTACGTAATGCCACTACGAATCAGTATTAACACCttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>TTTGCTAAAACCGATAGTTGCGCCGACAGCAGCAAATGAAAAttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>CCACCCTCACAGACGTTAGTAAATGAATAATATCAAACCCTCttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>ACAGTTAATTCAGGAGGTTTAGTACCGCACAGTTGAAAGGAAttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>CCGCCGCCAGGGTCAGTGCCTTGAGTAAGGAGCACTAACAACttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>GAATCAAGTCCCTCAGAGCCGCCACCAGACATTTGAGGATTTttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>CCAAAGACACCATCGATAGCAGCACCGTACAACTCGTATTAAttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>GAACAAAGTCAATCAATAGAAAATTCATAAAGTTTGAGTAACttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>CTTTACAGAGAAGCCCTTTTTAAGAAAACCAGAAGGAGCGGAttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>AACCTCCCGTTTTTGTTTAACGTCAAAAGATGGCAATTCATCttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>CATCCTAATTCCGGTATTCTAAGAACGCTTCTGAATAATGGAttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>GTAGGGCTTATAGATAAGTCCTGAACAATTTGCACGTAAAACttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>ATCGCAAGAAAATTCTTACCAGTATAAAGGTTTAACGTCAGAttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>ATATATGTGATATAACTATATGTAAATGTCGGGAGAAACAATttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>TCTGTAAATTAACAATTTCATTTTTTTAATGGAAACAAGTTACAAAATCttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 1, Side h5, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 2, Side h5, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 3, Side h5, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 4, Side h5, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 5, Side h5, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 6, Side h5, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 7, Side h5, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 8, Side h5, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 9, Side h5, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 10, Side h5, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 11, Side h5, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 12, Side h5, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 13, Side h5, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 14, Side h5, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 15, Side h5, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 16, Side h5, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 17, Side h5, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 18, Side h5, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 19, Side h5, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 20, Side h5, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 21, Side h5, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 22, Side h5, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 23, Side h5, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 24, Side h5, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 25, Side h5, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 26, Side h5, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 27, Side h5, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 28, Side h5, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 29, Side h5, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 30, Side h5, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 31, Side h5, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 32, Side h5, Cargo ID antiHomer</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3127,13 +3421,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -3171,7 +3473,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -3205,6 +3507,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -3239,9 +3542,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -3414,18 +3718,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E385"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="6.7109375" customWidth="1"/>
-    <col min="2" max="2" width="33.7109375" customWidth="1"/>
-    <col min="3" max="3" width="74.7109375" customWidth="1"/>
-    <col min="4" max="4" width="65.7109375" customWidth="1"/>
-    <col min="5" max="5" width="15.7109375" customWidth="1"/>
+    <col min="1" max="1" width="6.6640625" customWidth="1"/>
+    <col min="2" max="2" width="33.6640625" customWidth="1"/>
+    <col min="3" max="3" width="74.6640625" customWidth="1"/>
+    <col min="4" max="4" width="65.6640625" customWidth="1"/>
+    <col min="5" max="5" width="15.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3442,7 +3746,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -3459,7 +3763,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -3476,7 +3780,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -3493,7 +3797,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -3510,7 +3814,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -3527,7 +3831,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -3544,7 +3848,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -3561,7 +3865,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -3578,7 +3882,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -3595,7 +3899,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -3612,7 +3916,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>15</v>
       </c>
@@ -3629,7 +3933,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -3646,7 +3950,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>17</v>
       </c>
@@ -3663,7 +3967,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="15" spans="1:5">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>18</v>
       </c>
@@ -3680,7 +3984,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="16" spans="1:5">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>19</v>
       </c>
@@ -3697,7 +4001,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>20</v>
       </c>
@@ -3714,47 +4018,47 @@
         <v>500</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="22" spans="1:5">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="23" spans="1:5">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="24" spans="1:5">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="25" spans="1:5">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="26" spans="1:5">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>29</v>
       </c>
@@ -3771,7 +4075,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="27" spans="1:5">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>30</v>
       </c>
@@ -3788,7 +4092,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="28" spans="1:5">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>31</v>
       </c>
@@ -3805,7 +4109,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="29" spans="1:5">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>32</v>
       </c>
@@ -3822,7 +4126,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="30" spans="1:5">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>33</v>
       </c>
@@ -3839,7 +4143,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="31" spans="1:5">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>34</v>
       </c>
@@ -3856,7 +4160,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="32" spans="1:5">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>35</v>
       </c>
@@ -3873,7 +4177,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="33" spans="1:5">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>36</v>
       </c>
@@ -3890,7 +4194,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="34" spans="1:5">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>37</v>
       </c>
@@ -3907,7 +4211,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="35" spans="1:5">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>38</v>
       </c>
@@ -3924,7 +4228,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="36" spans="1:5">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>39</v>
       </c>
@@ -3941,7 +4245,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="37" spans="1:5">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>40</v>
       </c>
@@ -3958,7 +4262,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="38" spans="1:5">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>41</v>
       </c>
@@ -3975,7 +4279,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="39" spans="1:5">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>42</v>
       </c>
@@ -3992,7 +4296,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="40" spans="1:5">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>43</v>
       </c>
@@ -4009,7 +4313,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="41" spans="1:5">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>44</v>
       </c>
@@ -4026,47 +4330,47 @@
         <v>500</v>
       </c>
     </row>
-    <row r="42" spans="1:5">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="43" spans="1:5">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="44" spans="1:5">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="45" spans="1:5">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="46" spans="1:5">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="47" spans="1:5">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="48" spans="1:5">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="49" spans="1:5">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="50" spans="1:5">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>53</v>
       </c>
@@ -4083,7 +4387,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="51" spans="1:5">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>54</v>
       </c>
@@ -4100,7 +4404,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="52" spans="1:5">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>55</v>
       </c>
@@ -4117,7 +4421,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="53" spans="1:5">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>56</v>
       </c>
@@ -4134,7 +4438,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="54" spans="1:5">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>57</v>
       </c>
@@ -4151,7 +4455,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="55" spans="1:5">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>58</v>
       </c>
@@ -4168,7 +4472,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="56" spans="1:5">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>59</v>
       </c>
@@ -4185,7 +4489,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="57" spans="1:5">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>60</v>
       </c>
@@ -4202,7 +4506,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="58" spans="1:5">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>61</v>
       </c>
@@ -4219,7 +4523,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="59" spans="1:5">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>62</v>
       </c>
@@ -4236,7 +4540,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="60" spans="1:5">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>63</v>
       </c>
@@ -4253,7 +4557,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="61" spans="1:5">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>64</v>
       </c>
@@ -4270,7 +4574,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="62" spans="1:5">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>65</v>
       </c>
@@ -4287,7 +4591,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="63" spans="1:5">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>66</v>
       </c>
@@ -4304,7 +4608,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="64" spans="1:5">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>67</v>
       </c>
@@ -4321,7 +4625,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="65" spans="1:5">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>68</v>
       </c>
@@ -4338,47 +4642,47 @@
         <v>500</v>
       </c>
     </row>
-    <row r="66" spans="1:5">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="67" spans="1:5">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="68" spans="1:5">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="69" spans="1:5">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="70" spans="1:5">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="71" spans="1:5">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="72" spans="1:5">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="73" spans="1:5">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="74" spans="1:5">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>77</v>
       </c>
@@ -4395,7 +4699,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="75" spans="1:5">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>78</v>
       </c>
@@ -4412,7 +4716,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="76" spans="1:5">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>79</v>
       </c>
@@ -4429,7 +4733,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="77" spans="1:5">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>80</v>
       </c>
@@ -4446,7 +4750,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="78" spans="1:5">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>81</v>
       </c>
@@ -4463,7 +4767,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="79" spans="1:5">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>82</v>
       </c>
@@ -4480,7 +4784,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="80" spans="1:5">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>83</v>
       </c>
@@ -4497,7 +4801,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="81" spans="1:5">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>84</v>
       </c>
@@ -4514,7 +4818,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="82" spans="1:5">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>85</v>
       </c>
@@ -4531,7 +4835,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="83" spans="1:5">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>86</v>
       </c>
@@ -4548,7 +4852,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="84" spans="1:5">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>87</v>
       </c>
@@ -4565,7 +4869,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="85" spans="1:5">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>88</v>
       </c>
@@ -4582,7 +4886,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="86" spans="1:5">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>89</v>
       </c>
@@ -4599,7 +4903,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="87" spans="1:5">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>90</v>
       </c>
@@ -4616,7 +4920,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="88" spans="1:5">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>91</v>
       </c>
@@ -4633,7 +4937,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="89" spans="1:5">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>92</v>
       </c>
@@ -4650,47 +4954,47 @@
         <v>500</v>
       </c>
     </row>
-    <row r="90" spans="1:5">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="91" spans="1:5">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="92" spans="1:5">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="93" spans="1:5">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="94" spans="1:5">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="95" spans="1:5">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="96" spans="1:5">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="97" spans="1:5">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="98" spans="1:5">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>101</v>
       </c>
@@ -4707,7 +5011,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="99" spans="1:5">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>102</v>
       </c>
@@ -4724,7 +5028,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="100" spans="1:5">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>103</v>
       </c>
@@ -4741,7 +5045,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="101" spans="1:5">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>104</v>
       </c>
@@ -4758,7 +5062,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="102" spans="1:5">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>105</v>
       </c>
@@ -4775,7 +5079,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="103" spans="1:5">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>106</v>
       </c>
@@ -4792,7 +5096,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="104" spans="1:5">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>107</v>
       </c>
@@ -4809,7 +5113,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="105" spans="1:5">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>108</v>
       </c>
@@ -4826,7 +5130,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="106" spans="1:5">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>109</v>
       </c>
@@ -4843,7 +5147,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="107" spans="1:5">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>110</v>
       </c>
@@ -4860,7 +5164,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="108" spans="1:5">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>111</v>
       </c>
@@ -4877,7 +5181,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="109" spans="1:5">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>112</v>
       </c>
@@ -4894,7 +5198,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="110" spans="1:5">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>113</v>
       </c>
@@ -4911,7 +5215,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="111" spans="1:5">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>114</v>
       </c>
@@ -4928,7 +5232,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="112" spans="1:5">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>115</v>
       </c>
@@ -4945,7 +5249,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="113" spans="1:5">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>116</v>
       </c>
@@ -4962,47 +5266,47 @@
         <v>500</v>
       </c>
     </row>
-    <row r="114" spans="1:5">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="115" spans="1:5">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="116" spans="1:5">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="117" spans="1:5">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="118" spans="1:5">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="119" spans="1:5">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="120" spans="1:5">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="121" spans="1:5">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="122" spans="1:5">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>125</v>
       </c>
@@ -5019,7 +5323,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="123" spans="1:5">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
         <v>126</v>
       </c>
@@ -5036,7 +5340,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="124" spans="1:5">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
         <v>127</v>
       </c>
@@ -5053,7 +5357,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="125" spans="1:5">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
         <v>128</v>
       </c>
@@ -5070,7 +5374,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="126" spans="1:5">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
         <v>129</v>
       </c>
@@ -5087,7 +5391,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="127" spans="1:5">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
         <v>130</v>
       </c>
@@ -5104,7 +5408,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="128" spans="1:5">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
         <v>131</v>
       </c>
@@ -5121,7 +5425,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="129" spans="1:5">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
         <v>132</v>
       </c>
@@ -5138,7 +5442,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="130" spans="1:5">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
         <v>133</v>
       </c>
@@ -5155,7 +5459,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="131" spans="1:5">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
         <v>134</v>
       </c>
@@ -5172,7 +5476,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="132" spans="1:5">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
         <v>135</v>
       </c>
@@ -5189,7 +5493,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="133" spans="1:5">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
         <v>136</v>
       </c>
@@ -5206,7 +5510,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="134" spans="1:5">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
         <v>137</v>
       </c>
@@ -5223,7 +5527,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="135" spans="1:5">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
         <v>138</v>
       </c>
@@ -5240,7 +5544,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="136" spans="1:5">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
         <v>139</v>
       </c>
@@ -5257,7 +5561,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="137" spans="1:5">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
         <v>140</v>
       </c>
@@ -5274,47 +5578,47 @@
         <v>500</v>
       </c>
     </row>
-    <row r="138" spans="1:5">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="139" spans="1:5">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="140" spans="1:5">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="141" spans="1:5">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="142" spans="1:5">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="143" spans="1:5">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="144" spans="1:5">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="145" spans="1:5">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="146" spans="1:5">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
         <v>149</v>
       </c>
@@ -5331,7 +5635,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="147" spans="1:5">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
         <v>150</v>
       </c>
@@ -5348,7 +5652,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="148" spans="1:5">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A148" t="s">
         <v>151</v>
       </c>
@@ -5365,7 +5669,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="149" spans="1:5">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
         <v>152</v>
       </c>
@@ -5382,7 +5686,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="150" spans="1:5">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
         <v>153</v>
       </c>
@@ -5399,7 +5703,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="151" spans="1:5">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
         <v>154</v>
       </c>
@@ -5416,7 +5720,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="152" spans="1:5">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
         <v>155</v>
       </c>
@@ -5433,7 +5737,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="153" spans="1:5">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
         <v>156</v>
       </c>
@@ -5450,7 +5754,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="154" spans="1:5">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
         <v>157</v>
       </c>
@@ -5467,7 +5771,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="155" spans="1:5">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
         <v>158</v>
       </c>
@@ -5484,7 +5788,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="156" spans="1:5">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A156" t="s">
         <v>159</v>
       </c>
@@ -5501,7 +5805,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="157" spans="1:5">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
         <v>160</v>
       </c>
@@ -5518,7 +5822,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="158" spans="1:5">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
         <v>161</v>
       </c>
@@ -5535,7 +5839,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="159" spans="1:5">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
         <v>162</v>
       </c>
@@ -5552,7 +5856,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="160" spans="1:5">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
         <v>163</v>
       </c>
@@ -5569,7 +5873,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="161" spans="1:5">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A161" t="s">
         <v>164</v>
       </c>
@@ -5586,47 +5890,47 @@
         <v>500</v>
       </c>
     </row>
-    <row r="162" spans="1:5">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A162" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="163" spans="1:5">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A163" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="164" spans="1:5">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A164" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="165" spans="1:5">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="166" spans="1:5">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A166" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="167" spans="1:5">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A167" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="168" spans="1:5">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A168" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="169" spans="1:5">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A169" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="170" spans="1:5">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A170" t="s">
         <v>173</v>
       </c>
@@ -5643,7 +5947,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="171" spans="1:5">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A171" t="s">
         <v>174</v>
       </c>
@@ -5660,7 +5964,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="172" spans="1:5">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A172" t="s">
         <v>175</v>
       </c>
@@ -5677,7 +5981,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="173" spans="1:5">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A173" t="s">
         <v>176</v>
       </c>
@@ -5694,7 +5998,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="174" spans="1:5">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A174" t="s">
         <v>177</v>
       </c>
@@ -5711,7 +6015,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="175" spans="1:5">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A175" t="s">
         <v>178</v>
       </c>
@@ -5728,7 +6032,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="176" spans="1:5">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A176" t="s">
         <v>179</v>
       </c>
@@ -5745,7 +6049,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="177" spans="1:5">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
         <v>180</v>
       </c>
@@ -5762,7 +6066,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="178" spans="1:5">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
         <v>181</v>
       </c>
@@ -5779,7 +6083,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="179" spans="1:5">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A179" t="s">
         <v>182</v>
       </c>
@@ -5796,7 +6100,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="180" spans="1:5">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A180" t="s">
         <v>183</v>
       </c>
@@ -5813,7 +6117,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="181" spans="1:5">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A181" t="s">
         <v>184</v>
       </c>
@@ -5830,7 +6134,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="182" spans="1:5">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A182" t="s">
         <v>185</v>
       </c>
@@ -5847,7 +6151,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="183" spans="1:5">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A183" t="s">
         <v>186</v>
       </c>
@@ -5864,7 +6168,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="184" spans="1:5">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A184" t="s">
         <v>187</v>
       </c>
@@ -5881,7 +6185,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="185" spans="1:5">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A185" t="s">
         <v>188</v>
       </c>
@@ -5898,47 +6202,47 @@
         <v>500</v>
       </c>
     </row>
-    <row r="186" spans="1:5">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A186" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="187" spans="1:5">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A187" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="188" spans="1:5">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A188" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="189" spans="1:5">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A189" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="190" spans="1:5">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A190" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="191" spans="1:5">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A191" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="192" spans="1:5">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A192" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="193" spans="1:5">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A193" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="194" spans="1:5">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A194" t="s">
         <v>197</v>
       </c>
@@ -5955,7 +6259,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="195" spans="1:5">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A195" t="s">
         <v>198</v>
       </c>
@@ -5972,7 +6276,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="196" spans="1:5">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A196" t="s">
         <v>199</v>
       </c>
@@ -5989,7 +6293,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="197" spans="1:5">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A197" t="s">
         <v>200</v>
       </c>
@@ -6006,7 +6310,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="198" spans="1:5">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A198" t="s">
         <v>201</v>
       </c>
@@ -6023,7 +6327,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="199" spans="1:5">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A199" t="s">
         <v>202</v>
       </c>
@@ -6040,7 +6344,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="200" spans="1:5">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A200" t="s">
         <v>203</v>
       </c>
@@ -6057,7 +6361,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="201" spans="1:5">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A201" t="s">
         <v>204</v>
       </c>
@@ -6074,7 +6378,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="202" spans="1:5">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A202" t="s">
         <v>205</v>
       </c>
@@ -6091,7 +6395,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="203" spans="1:5">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A203" t="s">
         <v>206</v>
       </c>
@@ -6108,7 +6412,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="204" spans="1:5">
+    <row r="204" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A204" t="s">
         <v>207</v>
       </c>
@@ -6125,7 +6429,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="205" spans="1:5">
+    <row r="205" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A205" t="s">
         <v>208</v>
       </c>
@@ -6142,7 +6446,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="206" spans="1:5">
+    <row r="206" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A206" t="s">
         <v>209</v>
       </c>
@@ -6159,7 +6463,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="207" spans="1:5">
+    <row r="207" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A207" t="s">
         <v>210</v>
       </c>
@@ -6176,7 +6480,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="208" spans="1:5">
+    <row r="208" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A208" t="s">
         <v>211</v>
       </c>
@@ -6193,7 +6497,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="209" spans="1:5">
+    <row r="209" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A209" t="s">
         <v>212</v>
       </c>
@@ -6210,47 +6514,47 @@
         <v>500</v>
       </c>
     </row>
-    <row r="210" spans="1:5">
+    <row r="210" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A210" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="211" spans="1:5">
+    <row r="211" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A211" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="212" spans="1:5">
+    <row r="212" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A212" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="213" spans="1:5">
+    <row r="213" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A213" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="214" spans="1:5">
+    <row r="214" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A214" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="215" spans="1:5">
+    <row r="215" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A215" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="216" spans="1:5">
+    <row r="216" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A216" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="217" spans="1:5">
+    <row r="217" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A217" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="218" spans="1:5">
+    <row r="218" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A218" t="s">
         <v>221</v>
       </c>
@@ -6267,7 +6571,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="219" spans="1:5">
+    <row r="219" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A219" t="s">
         <v>222</v>
       </c>
@@ -6284,7 +6588,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="220" spans="1:5">
+    <row r="220" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A220" t="s">
         <v>223</v>
       </c>
@@ -6301,7 +6605,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="221" spans="1:5">
+    <row r="221" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A221" t="s">
         <v>224</v>
       </c>
@@ -6318,7 +6622,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="222" spans="1:5">
+    <row r="222" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A222" t="s">
         <v>225</v>
       </c>
@@ -6335,7 +6639,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="223" spans="1:5">
+    <row r="223" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A223" t="s">
         <v>226</v>
       </c>
@@ -6352,7 +6656,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="224" spans="1:5">
+    <row r="224" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A224" t="s">
         <v>227</v>
       </c>
@@ -6369,7 +6673,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="225" spans="1:5">
+    <row r="225" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A225" t="s">
         <v>228</v>
       </c>
@@ -6386,7 +6690,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="226" spans="1:5">
+    <row r="226" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A226" t="s">
         <v>229</v>
       </c>
@@ -6403,7 +6707,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="227" spans="1:5">
+    <row r="227" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A227" t="s">
         <v>230</v>
       </c>
@@ -6420,7 +6724,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="228" spans="1:5">
+    <row r="228" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A228" t="s">
         <v>231</v>
       </c>
@@ -6437,7 +6741,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="229" spans="1:5">
+    <row r="229" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A229" t="s">
         <v>232</v>
       </c>
@@ -6454,7 +6758,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="230" spans="1:5">
+    <row r="230" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A230" t="s">
         <v>233</v>
       </c>
@@ -6471,7 +6775,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="231" spans="1:5">
+    <row r="231" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A231" t="s">
         <v>234</v>
       </c>
@@ -6488,7 +6792,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="232" spans="1:5">
+    <row r="232" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A232" t="s">
         <v>235</v>
       </c>
@@ -6505,7 +6809,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="233" spans="1:5">
+    <row r="233" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A233" t="s">
         <v>236</v>
       </c>
@@ -6522,47 +6826,47 @@
         <v>500</v>
       </c>
     </row>
-    <row r="234" spans="1:5">
+    <row r="234" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A234" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="235" spans="1:5">
+    <row r="235" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A235" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="236" spans="1:5">
+    <row r="236" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A236" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="237" spans="1:5">
+    <row r="237" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A237" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="238" spans="1:5">
+    <row r="238" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A238" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="239" spans="1:5">
+    <row r="239" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A239" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="240" spans="1:5">
+    <row r="240" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A240" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="241" spans="1:5">
+    <row r="241" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A241" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="242" spans="1:5">
+    <row r="242" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A242" t="s">
         <v>245</v>
       </c>
@@ -6579,7 +6883,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="243" spans="1:5">
+    <row r="243" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A243" t="s">
         <v>246</v>
       </c>
@@ -6596,7 +6900,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="244" spans="1:5">
+    <row r="244" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A244" t="s">
         <v>247</v>
       </c>
@@ -6613,7 +6917,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="245" spans="1:5">
+    <row r="245" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A245" t="s">
         <v>248</v>
       </c>
@@ -6630,7 +6934,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="246" spans="1:5">
+    <row r="246" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A246" t="s">
         <v>249</v>
       </c>
@@ -6647,7 +6951,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="247" spans="1:5">
+    <row r="247" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A247" t="s">
         <v>250</v>
       </c>
@@ -6664,7 +6968,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="248" spans="1:5">
+    <row r="248" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A248" t="s">
         <v>251</v>
       </c>
@@ -6681,7 +6985,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="249" spans="1:5">
+    <row r="249" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A249" t="s">
         <v>252</v>
       </c>
@@ -6698,7 +7002,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="250" spans="1:5">
+    <row r="250" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A250" t="s">
         <v>253</v>
       </c>
@@ -6715,7 +7019,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="251" spans="1:5">
+    <row r="251" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A251" t="s">
         <v>254</v>
       </c>
@@ -6732,7 +7036,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="252" spans="1:5">
+    <row r="252" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A252" t="s">
         <v>255</v>
       </c>
@@ -6749,7 +7053,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="253" spans="1:5">
+    <row r="253" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A253" t="s">
         <v>256</v>
       </c>
@@ -6766,7 +7070,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="254" spans="1:5">
+    <row r="254" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A254" t="s">
         <v>257</v>
       </c>
@@ -6783,7 +7087,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="255" spans="1:5">
+    <row r="255" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A255" t="s">
         <v>258</v>
       </c>
@@ -6800,7 +7104,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="256" spans="1:5">
+    <row r="256" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A256" t="s">
         <v>259</v>
       </c>
@@ -6817,7 +7121,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="257" spans="1:5">
+    <row r="257" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A257" t="s">
         <v>260</v>
       </c>
@@ -6834,47 +7138,47 @@
         <v>500</v>
       </c>
     </row>
-    <row r="258" spans="1:5">
+    <row r="258" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A258" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="259" spans="1:5">
+    <row r="259" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A259" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="260" spans="1:5">
+    <row r="260" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A260" t="s">
         <v>263</v>
       </c>
     </row>
-    <row r="261" spans="1:5">
+    <row r="261" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A261" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="262" spans="1:5">
+    <row r="262" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A262" t="s">
         <v>265</v>
       </c>
     </row>
-    <row r="263" spans="1:5">
+    <row r="263" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A263" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="264" spans="1:5">
+    <row r="264" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A264" t="s">
         <v>267</v>
       </c>
     </row>
-    <row r="265" spans="1:5">
+    <row r="265" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A265" t="s">
         <v>268</v>
       </c>
     </row>
-    <row r="266" spans="1:5">
+    <row r="266" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A266" t="s">
         <v>269</v>
       </c>
@@ -6891,7 +7195,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="267" spans="1:5">
+    <row r="267" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A267" t="s">
         <v>270</v>
       </c>
@@ -6908,7 +7212,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="268" spans="1:5">
+    <row r="268" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A268" t="s">
         <v>271</v>
       </c>
@@ -6925,7 +7229,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="269" spans="1:5">
+    <row r="269" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A269" t="s">
         <v>272</v>
       </c>
@@ -6942,7 +7246,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="270" spans="1:5">
+    <row r="270" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A270" t="s">
         <v>273</v>
       </c>
@@ -6959,7 +7263,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="271" spans="1:5">
+    <row r="271" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A271" t="s">
         <v>274</v>
       </c>
@@ -6976,7 +7280,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="272" spans="1:5">
+    <row r="272" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A272" t="s">
         <v>275</v>
       </c>
@@ -6993,7 +7297,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="273" spans="1:5">
+    <row r="273" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A273" t="s">
         <v>276</v>
       </c>
@@ -7010,7 +7314,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="274" spans="1:5">
+    <row r="274" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A274" t="s">
         <v>277</v>
       </c>
@@ -7027,7 +7331,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="275" spans="1:5">
+    <row r="275" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A275" t="s">
         <v>278</v>
       </c>
@@ -7044,7 +7348,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="276" spans="1:5">
+    <row r="276" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A276" t="s">
         <v>279</v>
       </c>
@@ -7061,7 +7365,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="277" spans="1:5">
+    <row r="277" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A277" t="s">
         <v>280</v>
       </c>
@@ -7078,7 +7382,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="278" spans="1:5">
+    <row r="278" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A278" t="s">
         <v>281</v>
       </c>
@@ -7095,7 +7399,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="279" spans="1:5">
+    <row r="279" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A279" t="s">
         <v>282</v>
       </c>
@@ -7112,7 +7416,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="280" spans="1:5">
+    <row r="280" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A280" t="s">
         <v>283</v>
       </c>
@@ -7129,7 +7433,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="281" spans="1:5">
+    <row r="281" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A281" t="s">
         <v>284</v>
       </c>
@@ -7146,522 +7450,906 @@
         <v>500</v>
       </c>
     </row>
-    <row r="282" spans="1:5">
+    <row r="282" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A282" t="s">
         <v>285</v>
       </c>
     </row>
-    <row r="283" spans="1:5">
+    <row r="283" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A283" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="284" spans="1:5">
+    <row r="284" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A284" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="285" spans="1:5">
+    <row r="285" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A285" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="286" spans="1:5">
+    <row r="286" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A286" t="s">
         <v>289</v>
       </c>
     </row>
-    <row r="287" spans="1:5">
+    <row r="287" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A287" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="288" spans="1:5">
+    <row r="288" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A288" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="289" spans="1:1">
+    <row r="289" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A289" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="290" spans="1:1">
+    <row r="290" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A290" t="s">
         <v>293</v>
       </c>
     </row>
-    <row r="291" spans="1:1">
+    <row r="291" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A291" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="292" spans="1:1">
+    <row r="292" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A292" t="s">
         <v>295</v>
       </c>
     </row>
-    <row r="293" spans="1:1">
+    <row r="293" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A293" t="s">
         <v>296</v>
       </c>
     </row>
-    <row r="294" spans="1:1">
+    <row r="294" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A294" t="s">
         <v>297</v>
       </c>
     </row>
-    <row r="295" spans="1:1">
+    <row r="295" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A295" t="s">
         <v>298</v>
       </c>
     </row>
-    <row r="296" spans="1:1">
+    <row r="296" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A296" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="297" spans="1:1">
+    <row r="297" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A297" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="298" spans="1:1">
+    <row r="298" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A298" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="299" spans="1:1">
+    <row r="299" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A299" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="300" spans="1:1">
+    <row r="300" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A300" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="301" spans="1:1">
+    <row r="301" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A301" t="s">
         <v>304</v>
       </c>
     </row>
-    <row r="302" spans="1:1">
+    <row r="302" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A302" t="s">
         <v>305</v>
       </c>
     </row>
-    <row r="303" spans="1:1">
+    <row r="303" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A303" t="s">
         <v>306</v>
       </c>
     </row>
-    <row r="304" spans="1:1">
+    <row r="304" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A304" t="s">
         <v>307</v>
       </c>
     </row>
-    <row r="305" spans="1:1">
+    <row r="305" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A305" t="s">
         <v>308</v>
       </c>
     </row>
-    <row r="306" spans="1:1">
+    <row r="306" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A306" t="s">
         <v>309</v>
       </c>
     </row>
-    <row r="307" spans="1:1">
+    <row r="307" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A307" t="s">
         <v>310</v>
       </c>
     </row>
-    <row r="308" spans="1:1">
+    <row r="308" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A308" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="309" spans="1:1">
+    <row r="309" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A309" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="310" spans="1:1">
+    <row r="310" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A310" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="311" spans="1:1">
+    <row r="311" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A311" t="s">
         <v>314</v>
       </c>
     </row>
-    <row r="312" spans="1:1">
+    <row r="312" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A312" t="s">
         <v>315</v>
       </c>
     </row>
-    <row r="313" spans="1:1">
+    <row r="313" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A313" t="s">
         <v>316</v>
       </c>
     </row>
-    <row r="314" spans="1:1">
+    <row r="314" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A314" t="s">
         <v>317</v>
       </c>
     </row>
-    <row r="315" spans="1:1">
+    <row r="315" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A315" t="s">
         <v>318</v>
       </c>
     </row>
-    <row r="316" spans="1:1">
+    <row r="316" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A316" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="317" spans="1:1">
+    <row r="317" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A317" t="s">
         <v>320</v>
       </c>
     </row>
-    <row r="318" spans="1:1">
+    <row r="318" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A318" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="319" spans="1:1">
+    <row r="319" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A319" t="s">
         <v>322</v>
       </c>
     </row>
-    <row r="320" spans="1:1">
+    <row r="320" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A320" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="321" spans="1:1">
+    <row r="321" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A321" t="s">
         <v>324</v>
       </c>
     </row>
-    <row r="322" spans="1:1">
+    <row r="322" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A322" t="s">
         <v>325</v>
       </c>
     </row>
-    <row r="323" spans="1:1">
+    <row r="323" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A323" t="s">
         <v>326</v>
       </c>
     </row>
-    <row r="324" spans="1:1">
+    <row r="324" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A324" t="s">
         <v>327</v>
       </c>
     </row>
-    <row r="325" spans="1:1">
+    <row r="325" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A325" t="s">
         <v>328</v>
       </c>
     </row>
-    <row r="326" spans="1:1">
+    <row r="326" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A326" t="s">
         <v>329</v>
       </c>
     </row>
-    <row r="327" spans="1:1">
+    <row r="327" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A327" t="s">
         <v>330</v>
       </c>
     </row>
-    <row r="328" spans="1:1">
+    <row r="328" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A328" t="s">
         <v>331</v>
       </c>
     </row>
-    <row r="329" spans="1:1">
+    <row r="329" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A329" t="s">
         <v>332</v>
       </c>
     </row>
-    <row r="330" spans="1:1">
+    <row r="330" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A330" t="s">
         <v>333</v>
       </c>
     </row>
-    <row r="331" spans="1:1">
+    <row r="331" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A331" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="332" spans="1:1">
+    <row r="332" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A332" t="s">
         <v>335</v>
       </c>
     </row>
-    <row r="333" spans="1:1">
+    <row r="333" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A333" t="s">
         <v>336</v>
       </c>
     </row>
-    <row r="334" spans="1:1">
+    <row r="334" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A334" t="s">
         <v>337</v>
       </c>
     </row>
-    <row r="335" spans="1:1">
+    <row r="335" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A335" t="s">
         <v>338</v>
       </c>
     </row>
-    <row r="336" spans="1:1">
+    <row r="336" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A336" t="s">
         <v>339</v>
       </c>
     </row>
-    <row r="337" spans="1:1">
+    <row r="337" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A337" t="s">
         <v>340</v>
       </c>
     </row>
-    <row r="338" spans="1:1">
+    <row r="338" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A338" t="s">
         <v>341</v>
       </c>
-    </row>
-    <row r="339" spans="1:1">
+      <c r="B338" t="s">
+        <v>1007</v>
+      </c>
+      <c r="C338" t="s">
+        <v>1039</v>
+      </c>
+      <c r="D338" t="s">
+        <v>1071</v>
+      </c>
+      <c r="E338">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="339" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A339" t="s">
         <v>342</v>
       </c>
-    </row>
-    <row r="340" spans="1:1">
+      <c r="B339" t="s">
+        <v>1008</v>
+      </c>
+      <c r="C339" t="s">
+        <v>1040</v>
+      </c>
+      <c r="D339" t="s">
+        <v>1072</v>
+      </c>
+      <c r="E339">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="340" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A340" t="s">
         <v>343</v>
       </c>
-    </row>
-    <row r="341" spans="1:1">
+      <c r="B340" t="s">
+        <v>1009</v>
+      </c>
+      <c r="C340" t="s">
+        <v>1041</v>
+      </c>
+      <c r="D340" t="s">
+        <v>1073</v>
+      </c>
+      <c r="E340">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="341" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A341" t="s">
         <v>344</v>
       </c>
-    </row>
-    <row r="342" spans="1:1">
+      <c r="B341" t="s">
+        <v>1010</v>
+      </c>
+      <c r="C341" t="s">
+        <v>1042</v>
+      </c>
+      <c r="D341" t="s">
+        <v>1074</v>
+      </c>
+      <c r="E341">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="342" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A342" t="s">
         <v>345</v>
       </c>
-    </row>
-    <row r="343" spans="1:1">
+      <c r="B342" t="s">
+        <v>1011</v>
+      </c>
+      <c r="C342" t="s">
+        <v>1043</v>
+      </c>
+      <c r="D342" t="s">
+        <v>1075</v>
+      </c>
+      <c r="E342">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="343" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A343" t="s">
         <v>346</v>
       </c>
-    </row>
-    <row r="344" spans="1:1">
+      <c r="B343" t="s">
+        <v>1012</v>
+      </c>
+      <c r="C343" t="s">
+        <v>1044</v>
+      </c>
+      <c r="D343" t="s">
+        <v>1076</v>
+      </c>
+      <c r="E343">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="344" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A344" t="s">
         <v>347</v>
       </c>
-    </row>
-    <row r="345" spans="1:1">
+      <c r="B344" t="s">
+        <v>1013</v>
+      </c>
+      <c r="C344" t="s">
+        <v>1045</v>
+      </c>
+      <c r="D344" t="s">
+        <v>1077</v>
+      </c>
+      <c r="E344">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="345" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A345" t="s">
         <v>348</v>
       </c>
-    </row>
-    <row r="346" spans="1:1">
+      <c r="B345" t="s">
+        <v>1014</v>
+      </c>
+      <c r="C345" t="s">
+        <v>1046</v>
+      </c>
+      <c r="D345" t="s">
+        <v>1078</v>
+      </c>
+      <c r="E345">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="346" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A346" t="s">
         <v>349</v>
       </c>
-    </row>
-    <row r="347" spans="1:1">
+      <c r="B346" t="s">
+        <v>1015</v>
+      </c>
+      <c r="C346" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D346" t="s">
+        <v>1079</v>
+      </c>
+      <c r="E346">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="347" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A347" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="348" spans="1:1">
+      <c r="B347" t="s">
+        <v>1016</v>
+      </c>
+      <c r="C347" t="s">
+        <v>1048</v>
+      </c>
+      <c r="D347" t="s">
+        <v>1080</v>
+      </c>
+      <c r="E347">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="348" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A348" t="s">
         <v>351</v>
       </c>
-    </row>
-    <row r="349" spans="1:1">
+      <c r="B348" t="s">
+        <v>1017</v>
+      </c>
+      <c r="C348" t="s">
+        <v>1049</v>
+      </c>
+      <c r="D348" t="s">
+        <v>1081</v>
+      </c>
+      <c r="E348">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="349" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A349" t="s">
         <v>352</v>
       </c>
-    </row>
-    <row r="350" spans="1:1">
+      <c r="B349" t="s">
+        <v>1018</v>
+      </c>
+      <c r="C349" t="s">
+        <v>1050</v>
+      </c>
+      <c r="D349" t="s">
+        <v>1082</v>
+      </c>
+      <c r="E349">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="350" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A350" t="s">
         <v>353</v>
       </c>
-    </row>
-    <row r="351" spans="1:1">
+      <c r="B350" t="s">
+        <v>1019</v>
+      </c>
+      <c r="C350" t="s">
+        <v>1051</v>
+      </c>
+      <c r="D350" t="s">
+        <v>1083</v>
+      </c>
+      <c r="E350">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="351" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A351" t="s">
         <v>354</v>
       </c>
-    </row>
-    <row r="352" spans="1:1">
+      <c r="B351" t="s">
+        <v>1020</v>
+      </c>
+      <c r="C351" t="s">
+        <v>1052</v>
+      </c>
+      <c r="D351" t="s">
+        <v>1084</v>
+      </c>
+      <c r="E351">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="352" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A352" t="s">
         <v>355</v>
       </c>
-    </row>
-    <row r="353" spans="1:1">
+      <c r="B352" t="s">
+        <v>1021</v>
+      </c>
+      <c r="C352" t="s">
+        <v>1053</v>
+      </c>
+      <c r="D352" t="s">
+        <v>1085</v>
+      </c>
+      <c r="E352">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="353" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A353" t="s">
         <v>356</v>
       </c>
-    </row>
-    <row r="354" spans="1:1">
+      <c r="B353" t="s">
+        <v>1022</v>
+      </c>
+      <c r="C353" t="s">
+        <v>1054</v>
+      </c>
+      <c r="D353" t="s">
+        <v>1086</v>
+      </c>
+      <c r="E353">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="354" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A354" t="s">
         <v>357</v>
       </c>
     </row>
-    <row r="355" spans="1:1">
+    <row r="355" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A355" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="356" spans="1:1">
+    <row r="356" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A356" t="s">
         <v>359</v>
       </c>
     </row>
-    <row r="357" spans="1:1">
+    <row r="357" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A357" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="358" spans="1:1">
+    <row r="358" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A358" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="359" spans="1:1">
+    <row r="359" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A359" t="s">
         <v>362</v>
       </c>
     </row>
-    <row r="360" spans="1:1">
+    <row r="360" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A360" t="s">
         <v>363</v>
       </c>
     </row>
-    <row r="361" spans="1:1">
+    <row r="361" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A361" t="s">
         <v>364</v>
       </c>
     </row>
-    <row r="362" spans="1:1">
+    <row r="362" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A362" t="s">
         <v>365</v>
       </c>
-    </row>
-    <row r="363" spans="1:1">
+      <c r="B362" t="s">
+        <v>1023</v>
+      </c>
+      <c r="C362" t="s">
+        <v>1055</v>
+      </c>
+      <c r="D362" t="s">
+        <v>1087</v>
+      </c>
+      <c r="E362">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="363" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A363" t="s">
         <v>366</v>
       </c>
-    </row>
-    <row r="364" spans="1:1">
+      <c r="B363" t="s">
+        <v>1024</v>
+      </c>
+      <c r="C363" t="s">
+        <v>1056</v>
+      </c>
+      <c r="D363" t="s">
+        <v>1088</v>
+      </c>
+      <c r="E363">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="364" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A364" t="s">
         <v>367</v>
       </c>
-    </row>
-    <row r="365" spans="1:1">
+      <c r="B364" t="s">
+        <v>1025</v>
+      </c>
+      <c r="C364" t="s">
+        <v>1057</v>
+      </c>
+      <c r="D364" t="s">
+        <v>1089</v>
+      </c>
+      <c r="E364">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="365" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A365" t="s">
         <v>368</v>
       </c>
-    </row>
-    <row r="366" spans="1:1">
+      <c r="B365" t="s">
+        <v>1026</v>
+      </c>
+      <c r="C365" t="s">
+        <v>1058</v>
+      </c>
+      <c r="D365" t="s">
+        <v>1090</v>
+      </c>
+      <c r="E365">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="366" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A366" t="s">
         <v>369</v>
       </c>
-    </row>
-    <row r="367" spans="1:1">
+      <c r="B366" t="s">
+        <v>1027</v>
+      </c>
+      <c r="C366" t="s">
+        <v>1059</v>
+      </c>
+      <c r="D366" t="s">
+        <v>1091</v>
+      </c>
+      <c r="E366">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="367" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A367" t="s">
         <v>370</v>
       </c>
-    </row>
-    <row r="368" spans="1:1">
+      <c r="B367" t="s">
+        <v>1028</v>
+      </c>
+      <c r="C367" t="s">
+        <v>1060</v>
+      </c>
+      <c r="D367" t="s">
+        <v>1092</v>
+      </c>
+      <c r="E367">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="368" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A368" t="s">
         <v>371</v>
       </c>
-    </row>
-    <row r="369" spans="1:1">
+      <c r="B368" t="s">
+        <v>1029</v>
+      </c>
+      <c r="C368" t="s">
+        <v>1061</v>
+      </c>
+      <c r="D368" t="s">
+        <v>1093</v>
+      </c>
+      <c r="E368">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="369" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A369" t="s">
         <v>372</v>
       </c>
-    </row>
-    <row r="370" spans="1:1">
+      <c r="B369" t="s">
+        <v>1030</v>
+      </c>
+      <c r="C369" t="s">
+        <v>1062</v>
+      </c>
+      <c r="D369" t="s">
+        <v>1094</v>
+      </c>
+      <c r="E369">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="370" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A370" t="s">
         <v>373</v>
       </c>
-    </row>
-    <row r="371" spans="1:1">
+      <c r="B370" t="s">
+        <v>1031</v>
+      </c>
+      <c r="C370" t="s">
+        <v>1063</v>
+      </c>
+      <c r="D370" t="s">
+        <v>1095</v>
+      </c>
+      <c r="E370">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="371" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A371" t="s">
         <v>374</v>
       </c>
-    </row>
-    <row r="372" spans="1:1">
+      <c r="B371" t="s">
+        <v>1032</v>
+      </c>
+      <c r="C371" t="s">
+        <v>1064</v>
+      </c>
+      <c r="D371" t="s">
+        <v>1096</v>
+      </c>
+      <c r="E371">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="372" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A372" t="s">
         <v>375</v>
       </c>
-    </row>
-    <row r="373" spans="1:1">
+      <c r="B372" t="s">
+        <v>1033</v>
+      </c>
+      <c r="C372" t="s">
+        <v>1065</v>
+      </c>
+      <c r="D372" t="s">
+        <v>1097</v>
+      </c>
+      <c r="E372">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="373" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A373" t="s">
         <v>376</v>
       </c>
-    </row>
-    <row r="374" spans="1:1">
+      <c r="B373" t="s">
+        <v>1034</v>
+      </c>
+      <c r="C373" t="s">
+        <v>1066</v>
+      </c>
+      <c r="D373" t="s">
+        <v>1098</v>
+      </c>
+      <c r="E373">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="374" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A374" t="s">
         <v>377</v>
       </c>
-    </row>
-    <row r="375" spans="1:1">
+      <c r="B374" t="s">
+        <v>1035</v>
+      </c>
+      <c r="C374" t="s">
+        <v>1067</v>
+      </c>
+      <c r="D374" t="s">
+        <v>1099</v>
+      </c>
+      <c r="E374">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="375" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A375" t="s">
         <v>378</v>
       </c>
-    </row>
-    <row r="376" spans="1:1">
+      <c r="B375" t="s">
+        <v>1036</v>
+      </c>
+      <c r="C375" t="s">
+        <v>1068</v>
+      </c>
+      <c r="D375" t="s">
+        <v>1100</v>
+      </c>
+      <c r="E375">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="376" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A376" t="s">
         <v>379</v>
       </c>
-    </row>
-    <row r="377" spans="1:1">
+      <c r="B376" t="s">
+        <v>1037</v>
+      </c>
+      <c r="C376" t="s">
+        <v>1069</v>
+      </c>
+      <c r="D376" t="s">
+        <v>1101</v>
+      </c>
+      <c r="E376">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="377" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A377" t="s">
         <v>380</v>
       </c>
-    </row>
-    <row r="378" spans="1:1">
+      <c r="B377" t="s">
+        <v>1038</v>
+      </c>
+      <c r="C377" t="s">
+        <v>1070</v>
+      </c>
+      <c r="D377" t="s">
+        <v>1102</v>
+      </c>
+      <c r="E377">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="378" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A378" t="s">
         <v>381</v>
       </c>
     </row>
-    <row r="379" spans="1:1">
+    <row r="379" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A379" t="s">
         <v>382</v>
       </c>
     </row>
-    <row r="380" spans="1:1">
+    <row r="380" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A380" t="s">
         <v>383</v>
       </c>
     </row>
-    <row r="381" spans="1:1">
+    <row r="381" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A381" t="s">
         <v>384</v>
       </c>
     </row>
-    <row r="382" spans="1:1">
+    <row r="382" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A382" t="s">
         <v>385</v>
       </c>
     </row>
-    <row r="383" spans="1:1">
+    <row r="383" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A383" t="s">
         <v>386</v>
       </c>
     </row>
-    <row r="384" spans="1:1">
+    <row r="384" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A384" t="s">
         <v>387</v>
       </c>
     </row>
-    <row r="385" spans="1:1">
+    <row r="385" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A385" t="s">
         <v>388</v>
       </c>
@@ -7672,15 +8360,15 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Y17"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="16" width="33.7109375" customWidth="1"/>
-    <col min="17" max="24" width="5.7109375" customWidth="1"/>
+    <col min="1" max="16" width="33.6640625" customWidth="1"/>
+    <col min="17" max="24" width="5.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>989</v>
       </c>
@@ -7757,7 +8445,7 @@
         <v>988</v>
       </c>
     </row>
-    <row r="2" spans="1:25" s="2" customFormat="1">
+    <row r="2" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>990</v>
       </c>
@@ -7810,7 +8498,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="3" spans="1:25">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>991</v>
       </c>
@@ -7863,7 +8551,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="4" spans="1:25" s="2" customFormat="1">
+    <row r="4" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>992</v>
       </c>
@@ -7916,7 +8604,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="5" spans="1:25">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>993</v>
       </c>
@@ -7969,7 +8657,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="6" spans="1:25" s="2" customFormat="1">
+    <row r="6" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>994</v>
       </c>
@@ -8022,7 +8710,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="7" spans="1:25">
+    <row r="7" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>995</v>
       </c>
@@ -8075,7 +8763,7 @@
         <v>484</v>
       </c>
     </row>
-    <row r="8" spans="1:25" s="2" customFormat="1">
+    <row r="8" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>996</v>
       </c>
@@ -8128,7 +8816,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="9" spans="1:25">
+    <row r="9" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>997</v>
       </c>
@@ -8181,7 +8869,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="10" spans="1:25" s="2" customFormat="1">
+    <row r="10" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>998</v>
       </c>
@@ -8234,7 +8922,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="11" spans="1:25">
+    <row r="11" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>999</v>
       </c>
@@ -8287,7 +8975,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="12" spans="1:25" s="2" customFormat="1">
+    <row r="12" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>1000</v>
       </c>
@@ -8340,7 +9028,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="13" spans="1:25">
+    <row r="13" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>1001</v>
       </c>
@@ -8393,24 +9081,120 @@
         <v>580</v>
       </c>
     </row>
-    <row r="14" spans="1:25" s="2" customFormat="1">
+    <row r="14" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>1002</v>
       </c>
     </row>
-    <row r="15" spans="1:25">
+    <row r="15" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>1003</v>
       </c>
     </row>
-    <row r="16" spans="1:25" s="2" customFormat="1">
+    <row r="16" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>1004</v>
       </c>
-    </row>
-    <row r="17" spans="1:1">
+      <c r="B16" t="s">
+        <v>1007</v>
+      </c>
+      <c r="C16" t="s">
+        <v>1008</v>
+      </c>
+      <c r="D16" t="s">
+        <v>1009</v>
+      </c>
+      <c r="E16" t="s">
+        <v>1010</v>
+      </c>
+      <c r="F16" t="s">
+        <v>1011</v>
+      </c>
+      <c r="G16" t="s">
+        <v>1012</v>
+      </c>
+      <c r="H16" t="s">
+        <v>1013</v>
+      </c>
+      <c r="I16" t="s">
+        <v>1014</v>
+      </c>
+      <c r="J16" t="s">
+        <v>1015</v>
+      </c>
+      <c r="K16" t="s">
+        <v>1016</v>
+      </c>
+      <c r="L16" t="s">
+        <v>1017</v>
+      </c>
+      <c r="M16" t="s">
+        <v>1018</v>
+      </c>
+      <c r="N16" t="s">
+        <v>1019</v>
+      </c>
+      <c r="O16" t="s">
+        <v>1020</v>
+      </c>
+      <c r="P16" t="s">
+        <v>1021</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>1022</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>1005</v>
+      </c>
+      <c r="B17" t="s">
+        <v>1023</v>
+      </c>
+      <c r="C17" t="s">
+        <v>1024</v>
+      </c>
+      <c r="D17" t="s">
+        <v>1025</v>
+      </c>
+      <c r="E17" t="s">
+        <v>1026</v>
+      </c>
+      <c r="F17" t="s">
+        <v>1027</v>
+      </c>
+      <c r="G17" t="s">
+        <v>1028</v>
+      </c>
+      <c r="H17" t="s">
+        <v>1029</v>
+      </c>
+      <c r="I17" t="s">
+        <v>1030</v>
+      </c>
+      <c r="J17" t="s">
+        <v>1031</v>
+      </c>
+      <c r="K17" t="s">
+        <v>1032</v>
+      </c>
+      <c r="L17" t="s">
+        <v>1033</v>
+      </c>
+      <c r="M17" t="s">
+        <v>1034</v>
+      </c>
+      <c r="N17" t="s">
+        <v>1035</v>
+      </c>
+      <c r="O17" t="s">
+        <v>1036</v>
+      </c>
+      <c r="P17" t="s">
+        <v>1037</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>1038</v>
       </c>
     </row>
   </sheetData>
@@ -8419,15 +9203,15 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:Y17"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="9" width="3.7109375" customWidth="1"/>
-    <col min="10" max="24" width="4.7109375" customWidth="1"/>
+    <col min="1" max="9" width="3.6640625" customWidth="1"/>
+    <col min="10" max="24" width="4.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>989</v>
       </c>
@@ -8504,7 +9288,7 @@
         <v>988</v>
       </c>
     </row>
-    <row r="2" spans="1:25">
+    <row r="2" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>990</v>
       </c>
@@ -8581,7 +9365,7 @@
         <v>1006</v>
       </c>
     </row>
-    <row r="3" spans="1:25">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>991</v>
       </c>
@@ -8658,7 +9442,7 @@
         <v>1006</v>
       </c>
     </row>
-    <row r="4" spans="1:25">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>992</v>
       </c>
@@ -8735,7 +9519,7 @@
         <v>1006</v>
       </c>
     </row>
-    <row r="5" spans="1:25">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>993</v>
       </c>
@@ -8812,7 +9596,7 @@
         <v>1006</v>
       </c>
     </row>
-    <row r="6" spans="1:25">
+    <row r="6" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>994</v>
       </c>
@@ -8889,7 +9673,7 @@
         <v>1006</v>
       </c>
     </row>
-    <row r="7" spans="1:25">
+    <row r="7" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>995</v>
       </c>
@@ -8966,7 +9750,7 @@
         <v>1006</v>
       </c>
     </row>
-    <row r="8" spans="1:25">
+    <row r="8" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>996</v>
       </c>
@@ -9043,7 +9827,7 @@
         <v>1006</v>
       </c>
     </row>
-    <row r="9" spans="1:25">
+    <row r="9" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>997</v>
       </c>
@@ -9120,7 +9904,7 @@
         <v>1006</v>
       </c>
     </row>
-    <row r="10" spans="1:25">
+    <row r="10" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>998</v>
       </c>
@@ -9197,7 +9981,7 @@
         <v>1006</v>
       </c>
     </row>
-    <row r="11" spans="1:25">
+    <row r="11" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>999</v>
       </c>
@@ -9274,7 +10058,7 @@
         <v>1006</v>
       </c>
     </row>
-    <row r="12" spans="1:25">
+    <row r="12" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>1000</v>
       </c>
@@ -9351,7 +10135,7 @@
         <v>1006</v>
       </c>
     </row>
-    <row r="13" spans="1:25">
+    <row r="13" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>1001</v>
       </c>
@@ -9428,7 +10212,7 @@
         <v>1006</v>
       </c>
     </row>
-    <row r="14" spans="1:25">
+    <row r="14" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>1002</v>
       </c>
@@ -9505,7 +10289,7 @@
         <v>1006</v>
       </c>
     </row>
-    <row r="15" spans="1:25">
+    <row r="15" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>1003</v>
       </c>
@@ -9582,57 +10366,57 @@
         <v>1006</v>
       </c>
     </row>
-    <row r="16" spans="1:25">
+    <row r="16" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>1004</v>
       </c>
-      <c r="B16" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="G16" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="H16" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="I16" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="J16" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="K16" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="L16" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="M16" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="N16" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="O16" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="P16" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="Q16" s="4" t="s">
-        <v>1006</v>
+      <c r="B16" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="J16" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="K16" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="L16" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="M16" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="N16" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="O16" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="P16" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="Q16" s="3" t="s">
+        <v>992</v>
       </c>
       <c r="R16" s="4" t="s">
         <v>1006</v>
@@ -9659,57 +10443,57 @@
         <v>1006</v>
       </c>
     </row>
-    <row r="17" spans="1:25">
+    <row r="17" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>1005</v>
       </c>
-      <c r="B17" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="F17" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="G17" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="H17" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="I17" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="J17" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="K17" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="L17" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="M17" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="N17" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="O17" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="P17" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="Q17" s="4" t="s">
-        <v>1006</v>
+      <c r="B17" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="J17" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="K17" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="L17" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="M17" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="N17" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="O17" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="P17" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="Q17" s="3" t="s">
+        <v>992</v>
       </c>
       <c r="R17" s="4" t="s">
         <v>1006</v>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ mattaq31/Hash-CAD@642674dc31f8d5a81de1ce7db053fe84ce55dda6 🚀
</commit_message>
<xml_diff>
--- a/plates/cargo_plates/sw_src010_nelson_quimby_bart_edna_maxed.xlsx
+++ b/plates/cargo_plates/sw_src010_nelson_quimby_bart_edna_maxed.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/matt/Documents/Shih_Lab_Postdoc/research_projects/crisscross_code/crisscross_kit/crisscross/dna_source_plates/cargo_plates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27E4C657-E5B5-F345-BE7F-D15A67240173}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A720E82B-0AB8-3F48-BC33-AB810E517CD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="50440" windowHeight="28180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1751" uniqueCount="1103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1879" uniqueCount="1199">
   <si>
     <t>well</t>
   </si>
@@ -3331,6 +3331,294 @@
   </si>
   <si>
     <t>Cargo Handle For Slat Position 32, Side h5, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h2-position_1</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h2-position_2</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h2-position_3</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h2-position_4</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h2-position_5</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h2-position_6</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h2-position_7</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h2-position_8</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h2-position_9</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h2-position_10</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h2-position_11</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h2-position_12</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h2-position_13</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h2-position_14</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h2-position_15</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h2-position_16</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h2-position_17</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h2-position_18</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h2-position_19</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h2-position_20</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h2-position_21</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h2-position_22</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h2-position_23</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h2-position_24</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h2-position_25</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h2-position_26</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h2-position_27</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h2-position_28</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h2-position_29</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h2-position_30</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h2-position_31</t>
+  </si>
+  <si>
+    <t>CARGO-antiHomer-h2-position_32</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 1, Side h2, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 2, Side h2, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 3, Side h2, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 4, Side h2, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 5, Side h2, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 6, Side h2, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 7, Side h2, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 8, Side h2, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 9, Side h2, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 10, Side h2, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 11, Side h2, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 12, Side h2, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 13, Side h2, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 14, Side h2, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 15, Side h2, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 16, Side h2, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 17, Side h2, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 18, Side h2, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 19, Side h2, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 20, Side h2, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 21, Side h2, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 22, Side h2, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 23, Side h2, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 24, Side h2, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 25, Side h2, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 26, Side h2, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 27, Side h2, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 28, Side h2, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 29, Side h2, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 30, Side h2, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 31, Side h2, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 32, Side h2, Cargo ID antiHomer</t>
+  </si>
+  <si>
+    <t>GGGCGCCAGGGTGCTGGTTTGCCCCAGCAGGTTCCAGTTTGGttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>TAGCTGTTTCCTAGCTAACTCACATTAATTGGTTTGCGTATTttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>CAGCGGTGCCGGTTTCACGGTCATACCGGGTAATCATGGTCAttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>AACCAGCTTACGACTGTTGCCCTGCGGCTGGTTACCTGCAGCttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>CTTTAGTGATGACACATCCTCATAACGGAAGCCATCCCACGCttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>GAAACAATCGGCAAGAGACGCAGAAACAGCCGCACAGGCGGCttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>AAGCGCCATTCGGCAAGGCGATTAAGTTGGATAACCTCACCGttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>TCAACATTAAATGGCGCATCGTAACCGTGCGGAAACCAGGCAttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>TCGTAAAACTAGCGTTAATATTTTGTTAAAAGCCAGCTTTCAttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>TATTTTAAATGCCGTTCTAGCTGATAAATTGATGAACGGTAAttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>AGCTGAAAAGGTAGCCTCAGAGCATAAAGCAGAACCCTCATAttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>CATTTTTGCGGAATTCCATATAACAGTTGAATTTGGGGCGCGttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>AAACGAGAATGAGAAAGACTTCAAATATCGTTGATAAGAGGTttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>CCAAAAGGAATTAGAAGTTTTGCCAGAGGGAAACAGTTCAGAttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>TAAATTGGGCTTGGAAGAAAAATCTACGTTAGATACATAACGttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>CGAGGCGCAGACCTTCATCAAGAGTAATCTCAGAACGAGTAGttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>ATGAGGAAGTTTTCTTTGACCCCCAGCGATACTTAGCCGGAAttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>TTCGAGGTGAATGCTTGCAGGGAGTTAAAGAAAGACTTTTTCttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>CGTAACGATCTAGAGAATAGAAAGGAACAATATCAGCTTGCTttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>TATAGCCCGGAACCTCATTTTCAGGGATAGCCTCATAGTTAGttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>CAGGAGTGTACTTATTCTGAAACATGAAAGGGTTGATATAAGttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>CCTCAGAACCGCCAGACGATTGGCCTTGATCTTTTGATGATAttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>TAGCAAGGCCGGCGTTTTCATCGGCATTTTCAGAGCCGCCACttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>AGACACCACGGAGGAGGGAAGGTAAATATTCACCATTACCATttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>AACAATGAAATAAATAATAACGGAATACCCAAAGAAACGCAAttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>TATTTATCCCAAGCATTAGACGGGAGAATTATAAGAGCAAGAttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>TAGCAAGCAAATAATCAAGATTAGTTGCTAAAACAGCCATATttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>CTAATGCAGAACTAATCGGCTGTCTTTCCTTACCGCGCCCAAttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>AAGCCTGTTTAGCGCCAACATGTAATTTAGCAACATGTTCAGttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>CCTTTTTAACCTAATATATTTTAGTTAATTAATTACTAGAAAttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>ATTAATTACATTCGTCGCTATTAATTAATTTCTGAGAGACTAttACAACCCCTAATATCTTTCCT</t>
+  </si>
+  <si>
+    <t>CTTGAAAACATAGATGATGAAACAAAACAAAttACAACCCCTAATATCTTTCCT</t>
   </si>
 </sst>
 </file>
@@ -3717,6 +4005,28 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="0">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{9E3C4801-77B8-C140-9F30-07E6D70842C2}">
+  <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;d4553de9-24ec-4352-a3aa-5111030725a3&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E385"/>
@@ -7485,242 +7795,626 @@
         <v>291</v>
       </c>
     </row>
-    <row r="289" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="289" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A289" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="290" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="290" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A290" t="s">
         <v>293</v>
       </c>
-    </row>
-    <row r="291" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B290" t="s">
+        <v>1103</v>
+      </c>
+      <c r="C290" t="s">
+        <v>1167</v>
+      </c>
+      <c r="D290" t="s">
+        <v>1135</v>
+      </c>
+      <c r="E290">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="291" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A291" t="s">
         <v>294</v>
       </c>
-    </row>
-    <row r="292" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B291" t="s">
+        <v>1104</v>
+      </c>
+      <c r="C291" t="s">
+        <v>1168</v>
+      </c>
+      <c r="D291" t="s">
+        <v>1136</v>
+      </c>
+      <c r="E291">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="292" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A292" t="s">
         <v>295</v>
       </c>
-    </row>
-    <row r="293" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B292" t="s">
+        <v>1105</v>
+      </c>
+      <c r="C292" t="s">
+        <v>1169</v>
+      </c>
+      <c r="D292" t="s">
+        <v>1137</v>
+      </c>
+      <c r="E292">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="293" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A293" t="s">
         <v>296</v>
       </c>
-    </row>
-    <row r="294" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B293" t="s">
+        <v>1106</v>
+      </c>
+      <c r="C293" t="s">
+        <v>1170</v>
+      </c>
+      <c r="D293" t="s">
+        <v>1138</v>
+      </c>
+      <c r="E293">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="294" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A294" t="s">
         <v>297</v>
       </c>
-    </row>
-    <row r="295" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B294" t="s">
+        <v>1107</v>
+      </c>
+      <c r="C294" t="s">
+        <v>1171</v>
+      </c>
+      <c r="D294" t="s">
+        <v>1139</v>
+      </c>
+      <c r="E294">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="295" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A295" t="s">
         <v>298</v>
       </c>
-    </row>
-    <row r="296" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B295" t="s">
+        <v>1108</v>
+      </c>
+      <c r="C295" t="s">
+        <v>1172</v>
+      </c>
+      <c r="D295" t="s">
+        <v>1140</v>
+      </c>
+      <c r="E295">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="296" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A296" t="s">
         <v>299</v>
       </c>
-    </row>
-    <row r="297" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B296" t="s">
+        <v>1109</v>
+      </c>
+      <c r="C296" t="s">
+        <v>1173</v>
+      </c>
+      <c r="D296" t="s">
+        <v>1141</v>
+      </c>
+      <c r="E296">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="297" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A297" t="s">
         <v>300</v>
       </c>
-    </row>
-    <row r="298" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B297" t="s">
+        <v>1110</v>
+      </c>
+      <c r="C297" t="s">
+        <v>1174</v>
+      </c>
+      <c r="D297" t="s">
+        <v>1142</v>
+      </c>
+      <c r="E297">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="298" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A298" t="s">
         <v>301</v>
       </c>
-    </row>
-    <row r="299" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B298" t="s">
+        <v>1111</v>
+      </c>
+      <c r="C298" t="s">
+        <v>1175</v>
+      </c>
+      <c r="D298" t="s">
+        <v>1143</v>
+      </c>
+      <c r="E298">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="299" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A299" t="s">
         <v>302</v>
       </c>
-    </row>
-    <row r="300" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B299" t="s">
+        <v>1112</v>
+      </c>
+      <c r="C299" t="s">
+        <v>1176</v>
+      </c>
+      <c r="D299" t="s">
+        <v>1144</v>
+      </c>
+      <c r="E299">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="300" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A300" t="s">
         <v>303</v>
       </c>
-    </row>
-    <row r="301" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B300" t="s">
+        <v>1113</v>
+      </c>
+      <c r="C300" t="s">
+        <v>1177</v>
+      </c>
+      <c r="D300" t="s">
+        <v>1145</v>
+      </c>
+      <c r="E300">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="301" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A301" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="302" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B301" t="s">
+        <v>1114</v>
+      </c>
+      <c r="C301" t="s">
+        <v>1178</v>
+      </c>
+      <c r="D301" t="s">
+        <v>1146</v>
+      </c>
+      <c r="E301">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="302" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A302" t="s">
         <v>305</v>
       </c>
-    </row>
-    <row r="303" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B302" t="s">
+        <v>1115</v>
+      </c>
+      <c r="C302" t="s">
+        <v>1179</v>
+      </c>
+      <c r="D302" t="s">
+        <v>1147</v>
+      </c>
+      <c r="E302">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="303" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A303" t="s">
         <v>306</v>
       </c>
-    </row>
-    <row r="304" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B303" t="s">
+        <v>1116</v>
+      </c>
+      <c r="C303" t="s">
+        <v>1180</v>
+      </c>
+      <c r="D303" t="s">
+        <v>1148</v>
+      </c>
+      <c r="E303">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="304" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A304" t="s">
         <v>307</v>
       </c>
-    </row>
-    <row r="305" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B304" t="s">
+        <v>1117</v>
+      </c>
+      <c r="C304" t="s">
+        <v>1181</v>
+      </c>
+      <c r="D304" t="s">
+        <v>1149</v>
+      </c>
+      <c r="E304">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="305" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A305" t="s">
         <v>308</v>
       </c>
-    </row>
-    <row r="306" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B305" t="s">
+        <v>1118</v>
+      </c>
+      <c r="C305" t="s">
+        <v>1182</v>
+      </c>
+      <c r="D305" t="s">
+        <v>1150</v>
+      </c>
+      <c r="E305">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="306" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A306" t="s">
         <v>309</v>
       </c>
     </row>
-    <row r="307" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="307" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A307" t="s">
         <v>310</v>
       </c>
     </row>
-    <row r="308" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="308" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A308" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="309" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="309" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A309" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="310" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="310" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A310" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="311" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="311" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A311" t="s">
         <v>314</v>
       </c>
     </row>
-    <row r="312" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="312" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A312" t="s">
         <v>315</v>
       </c>
     </row>
-    <row r="313" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="313" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A313" t="s">
         <v>316</v>
       </c>
     </row>
-    <row r="314" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="314" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A314" t="s">
         <v>317</v>
       </c>
-    </row>
-    <row r="315" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B314" t="s">
+        <v>1119</v>
+      </c>
+      <c r="C314" t="s">
+        <v>1183</v>
+      </c>
+      <c r="D314" t="s">
+        <v>1151</v>
+      </c>
+      <c r="E314">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="315" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A315" t="s">
         <v>318</v>
       </c>
-    </row>
-    <row r="316" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B315" t="s">
+        <v>1120</v>
+      </c>
+      <c r="C315" t="s">
+        <v>1184</v>
+      </c>
+      <c r="D315" t="s">
+        <v>1152</v>
+      </c>
+      <c r="E315">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="316" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A316" t="s">
         <v>319</v>
       </c>
-    </row>
-    <row r="317" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B316" t="s">
+        <v>1121</v>
+      </c>
+      <c r="C316" t="s">
+        <v>1185</v>
+      </c>
+      <c r="D316" t="s">
+        <v>1153</v>
+      </c>
+      <c r="E316">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="317" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A317" t="s">
         <v>320</v>
       </c>
-    </row>
-    <row r="318" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B317" t="s">
+        <v>1122</v>
+      </c>
+      <c r="C317" t="s">
+        <v>1186</v>
+      </c>
+      <c r="D317" t="s">
+        <v>1154</v>
+      </c>
+      <c r="E317">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="318" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A318" t="s">
         <v>321</v>
       </c>
-    </row>
-    <row r="319" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B318" t="s">
+        <v>1123</v>
+      </c>
+      <c r="C318" t="s">
+        <v>1187</v>
+      </c>
+      <c r="D318" t="s">
+        <v>1155</v>
+      </c>
+      <c r="E318">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="319" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A319" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="320" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B319" t="s">
+        <v>1124</v>
+      </c>
+      <c r="C319" t="s">
+        <v>1188</v>
+      </c>
+      <c r="D319" t="s">
+        <v>1156</v>
+      </c>
+      <c r="E319">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="320" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A320" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="321" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B320" t="s">
+        <v>1125</v>
+      </c>
+      <c r="C320" t="s">
+        <v>1189</v>
+      </c>
+      <c r="D320" t="s">
+        <v>1157</v>
+      </c>
+      <c r="E320">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="321" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A321" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="322" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B321" t="s">
+        <v>1126</v>
+      </c>
+      <c r="C321" t="s">
+        <v>1190</v>
+      </c>
+      <c r="D321" t="s">
+        <v>1158</v>
+      </c>
+      <c r="E321">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="322" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A322" t="s">
         <v>325</v>
       </c>
-    </row>
-    <row r="323" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B322" t="s">
+        <v>1127</v>
+      </c>
+      <c r="C322" t="s">
+        <v>1191</v>
+      </c>
+      <c r="D322" t="s">
+        <v>1159</v>
+      </c>
+      <c r="E322">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="323" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A323" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="324" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B323" t="s">
+        <v>1128</v>
+      </c>
+      <c r="C323" t="s">
+        <v>1192</v>
+      </c>
+      <c r="D323" t="s">
+        <v>1160</v>
+      </c>
+      <c r="E323">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="324" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A324" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="325" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B324" t="s">
+        <v>1129</v>
+      </c>
+      <c r="C324" t="s">
+        <v>1193</v>
+      </c>
+      <c r="D324" t="s">
+        <v>1161</v>
+      </c>
+      <c r="E324">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="325" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A325" t="s">
         <v>328</v>
       </c>
-    </row>
-    <row r="326" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B325" t="s">
+        <v>1130</v>
+      </c>
+      <c r="C325" t="s">
+        <v>1194</v>
+      </c>
+      <c r="D325" t="s">
+        <v>1162</v>
+      </c>
+      <c r="E325">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="326" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A326" t="s">
         <v>329</v>
       </c>
-    </row>
-    <row r="327" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B326" t="s">
+        <v>1131</v>
+      </c>
+      <c r="C326" t="s">
+        <v>1195</v>
+      </c>
+      <c r="D326" t="s">
+        <v>1163</v>
+      </c>
+      <c r="E326">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="327" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A327" t="s">
         <v>330</v>
       </c>
-    </row>
-    <row r="328" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B327" t="s">
+        <v>1132</v>
+      </c>
+      <c r="C327" t="s">
+        <v>1196</v>
+      </c>
+      <c r="D327" t="s">
+        <v>1164</v>
+      </c>
+      <c r="E327">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="328" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A328" t="s">
         <v>331</v>
       </c>
-    </row>
-    <row r="329" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B328" t="s">
+        <v>1133</v>
+      </c>
+      <c r="C328" t="s">
+        <v>1197</v>
+      </c>
+      <c r="D328" t="s">
+        <v>1165</v>
+      </c>
+      <c r="E328">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="329" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A329" t="s">
         <v>332</v>
       </c>
-    </row>
-    <row r="330" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B329" t="s">
+        <v>1134</v>
+      </c>
+      <c r="C329" t="s">
+        <v>1198</v>
+      </c>
+      <c r="D329" t="s">
+        <v>1166</v>
+      </c>
+      <c r="E329">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="330" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A330" t="s">
         <v>333</v>
       </c>
     </row>
-    <row r="331" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="331" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A331" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="332" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="332" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A332" t="s">
         <v>335</v>
       </c>
     </row>
-    <row r="333" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="333" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A333" t="s">
         <v>336</v>
       </c>
     </row>
-    <row r="334" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="334" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A334" t="s">
         <v>337</v>
       </c>
     </row>
-    <row r="335" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="335" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A335" t="s">
         <v>338</v>
       </c>
     </row>
-    <row r="336" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="336" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A336" t="s">
         <v>339</v>
       </c>
@@ -9085,10 +9779,106 @@
       <c r="A14" s="1" t="s">
         <v>1002</v>
       </c>
+      <c r="B14" t="s">
+        <v>1103</v>
+      </c>
+      <c r="C14" t="s">
+        <v>1104</v>
+      </c>
+      <c r="D14" t="s">
+        <v>1105</v>
+      </c>
+      <c r="E14" t="s">
+        <v>1106</v>
+      </c>
+      <c r="F14" t="s">
+        <v>1107</v>
+      </c>
+      <c r="G14" t="s">
+        <v>1108</v>
+      </c>
+      <c r="H14" t="s">
+        <v>1109</v>
+      </c>
+      <c r="I14" t="s">
+        <v>1110</v>
+      </c>
+      <c r="J14" t="s">
+        <v>1111</v>
+      </c>
+      <c r="K14" t="s">
+        <v>1112</v>
+      </c>
+      <c r="L14" t="s">
+        <v>1113</v>
+      </c>
+      <c r="M14" t="s">
+        <v>1114</v>
+      </c>
+      <c r="N14" t="s">
+        <v>1115</v>
+      </c>
+      <c r="O14" t="s">
+        <v>1116</v>
+      </c>
+      <c r="P14" t="s">
+        <v>1117</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>1118</v>
+      </c>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>1003</v>
+      </c>
+      <c r="B15" t="s">
+        <v>1119</v>
+      </c>
+      <c r="C15" t="s">
+        <v>1120</v>
+      </c>
+      <c r="D15" t="s">
+        <v>1121</v>
+      </c>
+      <c r="E15" t="s">
+        <v>1122</v>
+      </c>
+      <c r="F15" t="s">
+        <v>1123</v>
+      </c>
+      <c r="G15" t="s">
+        <v>1124</v>
+      </c>
+      <c r="H15" t="s">
+        <v>1125</v>
+      </c>
+      <c r="I15" t="s">
+        <v>1126</v>
+      </c>
+      <c r="J15" t="s">
+        <v>1127</v>
+      </c>
+      <c r="K15" t="s">
+        <v>1128</v>
+      </c>
+      <c r="L15" t="s">
+        <v>1129</v>
+      </c>
+      <c r="M15" t="s">
+        <v>1130</v>
+      </c>
+      <c r="N15" t="s">
+        <v>1131</v>
+      </c>
+      <c r="O15" t="s">
+        <v>1132</v>
+      </c>
+      <c r="P15" t="s">
+        <v>1133</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>1134</v>
       </c>
     </row>
     <row r="16" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.2">
@@ -10216,53 +11006,53 @@
       <c r="A14" s="1" t="s">
         <v>1002</v>
       </c>
-      <c r="B14" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="H14" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="I14" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="J14" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="K14" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="L14" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="M14" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="N14" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="O14" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="P14" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="Q14" s="4" t="s">
-        <v>1006</v>
+      <c r="B14" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="K14" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="L14" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="M14" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="N14" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="O14" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="P14" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="Q14" s="3" t="s">
+        <v>992</v>
       </c>
       <c r="R14" s="4" t="s">
         <v>1006</v>
@@ -10293,53 +11083,53 @@
       <c r="A15" s="1" t="s">
         <v>1003</v>
       </c>
-      <c r="B15" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="G15" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="H15" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="I15" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="J15" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="K15" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="L15" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="M15" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="N15" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="O15" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="P15" s="4" t="s">
-        <v>1006</v>
-      </c>
-      <c r="Q15" s="4" t="s">
-        <v>1006</v>
+      <c r="B15" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="K15" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="L15" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="M15" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="N15" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="O15" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="P15" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="Q15" s="3" t="s">
+        <v>992</v>
       </c>
       <c r="R15" s="4" t="s">
         <v>1006</v>

</xml_diff>